<commit_message>
Updated login details using uipath
</commit_message>
<xml_diff>
--- a/Uipath.xlsx
+++ b/Uipath.xlsx
@@ -5,15 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yaswanth Asapu\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yaswanth Asapu\Documents\UiPath\iVIS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E8389D8-A3D4-496C-9C6E-E9746305FAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BE96391-BC03-4C63-A57D-EDDB6DABF185}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet-2" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="316">
   <si>
     <t>mohammad.yakub91k@gmail.com</t>
   </si>
@@ -931,13 +932,55 @@
   </si>
   <si>
     <t>Ivis@1234</t>
+  </si>
+  <si>
+    <t>vivek.r@ivis.net</t>
+  </si>
+  <si>
+    <t>Ivis@123</t>
+  </si>
+  <si>
+    <t>adithya.karpuram@ivis.net</t>
+  </si>
+  <si>
+    <t>teja.v@ivis.net</t>
+  </si>
+  <si>
+    <t>rathikanth.d@ivis.net</t>
+  </si>
+  <si>
+    <t>ticketanalysis@ivis.net</t>
+  </si>
+  <si>
+    <t>ivisfm@ivis.net</t>
+  </si>
+  <si>
+    <t>umashankar</t>
+  </si>
+  <si>
+    <t>IV2222</t>
+  </si>
+  <si>
+    <t>malathi.b@ivis.net</t>
+  </si>
+  <si>
+    <t>ship@ivis.net</t>
+  </si>
+  <si>
+    <t>returns@ivis.net</t>
+  </si>
+  <si>
+    <t>charan.v@ivis.net</t>
+  </si>
+  <si>
+    <t>syamprasad.m@ivis.net</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -959,6 +1002,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1026,11 +1075,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1312,13 +1362,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B300"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="41.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.28515625" customWidth="1"/>
+    <col min="1" max="1" width="41.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>299</v>
       </c>
@@ -1326,7 +1376,7 @@
         <v>300</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1334,7 +1384,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -1342,7 +1392,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
@@ -1350,7 +1400,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
@@ -1358,7 +1408,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -1366,7 +1416,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>5</v>
       </c>
@@ -1374,7 +1424,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>6</v>
       </c>
@@ -1382,7 +1432,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>7</v>
       </c>
@@ -1390,7 +1440,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>8</v>
       </c>
@@ -1398,7 +1448,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
@@ -1406,7 +1456,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>10</v>
       </c>
@@ -1414,7 +1464,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>11</v>
       </c>
@@ -1422,7 +1472,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>12</v>
       </c>
@@ -1430,7 +1480,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>13</v>
       </c>
@@ -1438,7 +1488,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>14</v>
       </c>
@@ -1446,7 +1496,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>15</v>
       </c>
@@ -1454,7 +1504,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>16</v>
       </c>
@@ -1462,7 +1512,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>17</v>
       </c>
@@ -1470,7 +1520,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>18</v>
       </c>
@@ -1478,7 +1528,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>19</v>
       </c>
@@ -1486,7 +1536,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>20</v>
       </c>
@@ -1494,7 +1544,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>21</v>
       </c>
@@ -1502,7 +1552,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>22</v>
       </c>
@@ -1510,7 +1560,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>23</v>
       </c>
@@ -1518,7 +1568,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>24</v>
       </c>
@@ -1526,7 +1576,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>25</v>
       </c>
@@ -1534,7 +1584,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>26</v>
       </c>
@@ -1542,7 +1592,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>27</v>
       </c>
@@ -1550,7 +1600,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>28</v>
       </c>
@@ -1558,7 +1608,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>29</v>
       </c>
@@ -1566,7 +1616,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>30</v>
       </c>
@@ -1574,7 +1624,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>31</v>
       </c>
@@ -1582,7 +1632,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>32</v>
       </c>
@@ -1590,7 +1640,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>33</v>
       </c>
@@ -1598,7 +1648,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>34</v>
       </c>
@@ -1606,7 +1656,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>35</v>
       </c>
@@ -1614,7 +1664,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>36</v>
       </c>
@@ -1622,7 +1672,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>37</v>
       </c>
@@ -1630,7 +1680,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>38</v>
       </c>
@@ -1638,7 +1688,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>39</v>
       </c>
@@ -1646,7 +1696,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>40</v>
       </c>
@@ -1654,7 +1704,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>41</v>
       </c>
@@ -1662,7 +1712,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>42</v>
       </c>
@@ -1670,7 +1720,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>43</v>
       </c>
@@ -1678,7 +1728,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>44</v>
       </c>
@@ -1686,7 +1736,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>45</v>
       </c>
@@ -1694,7 +1744,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>46</v>
       </c>
@@ -1702,7 +1752,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>47</v>
       </c>
@@ -1710,7 +1760,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>48</v>
       </c>
@@ -1718,7 +1768,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>49</v>
       </c>
@@ -1726,7 +1776,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>50</v>
       </c>
@@ -1734,7 +1784,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>51</v>
       </c>
@@ -1742,7 +1792,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>52</v>
       </c>
@@ -1750,7 +1800,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>53</v>
       </c>
@@ -1758,7 +1808,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>54</v>
       </c>
@@ -1766,7 +1816,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>55</v>
       </c>
@@ -1774,7 +1824,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>56</v>
       </c>
@@ -1782,7 +1832,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>57</v>
       </c>
@@ -1790,7 +1840,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>58</v>
       </c>
@@ -1798,7 +1848,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>59</v>
       </c>
@@ -1806,7 +1856,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>60</v>
       </c>
@@ -1814,7 +1864,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>61</v>
       </c>
@@ -1822,7 +1872,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>62</v>
       </c>
@@ -1830,7 +1880,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>63</v>
       </c>
@@ -1838,7 +1888,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>64</v>
       </c>
@@ -1846,7 +1896,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>65</v>
       </c>
@@ -1854,7 +1904,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>66</v>
       </c>
@@ -1862,7 +1912,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>67</v>
       </c>
@@ -1870,7 +1920,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>68</v>
       </c>
@@ -1878,7 +1928,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>69</v>
       </c>
@@ -1886,7 +1936,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>70</v>
       </c>
@@ -1894,7 +1944,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>71</v>
       </c>
@@ -1902,7 +1952,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>72</v>
       </c>
@@ -1910,7 +1960,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>73</v>
       </c>
@@ -1918,7 +1968,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>74</v>
       </c>
@@ -1926,7 +1976,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>75</v>
       </c>
@@ -1934,7 +1984,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>76</v>
       </c>
@@ -1942,7 +1992,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>77</v>
       </c>
@@ -1950,7 +2000,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A80" s="2" t="s">
         <v>78</v>
       </c>
@@ -1958,7 +2008,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A81" s="2" t="s">
         <v>79</v>
       </c>
@@ -1966,7 +2016,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A82" s="2" t="s">
         <v>80</v>
       </c>
@@ -1974,7 +2024,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A83" s="2" t="s">
         <v>81</v>
       </c>
@@ -1982,7 +2032,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A84" s="2" t="s">
         <v>82</v>
       </c>
@@ -1990,7 +2040,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A85" s="2" t="s">
         <v>83</v>
       </c>
@@ -1998,7 +2048,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A86" s="2" t="s">
         <v>84</v>
       </c>
@@ -2006,7 +2056,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A87" s="2" t="s">
         <v>85</v>
       </c>
@@ -2014,7 +2064,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A88" s="2" t="s">
         <v>86</v>
       </c>
@@ -2022,7 +2072,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A89" s="2" t="s">
         <v>87</v>
       </c>
@@ -2030,7 +2080,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A90" s="2" t="s">
         <v>88</v>
       </c>
@@ -2038,7 +2088,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A91" s="2" t="s">
         <v>89</v>
       </c>
@@ -2046,7 +2096,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A92" s="2" t="s">
         <v>90</v>
       </c>
@@ -2054,7 +2104,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A93" s="2" t="s">
         <v>91</v>
       </c>
@@ -2062,7 +2112,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A94" s="2" t="s">
         <v>92</v>
       </c>
@@ -2070,7 +2120,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A95" s="2" t="s">
         <v>93</v>
       </c>
@@ -2078,7 +2128,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A96" s="2" t="s">
         <v>94</v>
       </c>
@@ -2086,7 +2136,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A97" s="2" t="s">
         <v>95</v>
       </c>
@@ -2094,7 +2144,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A98" s="2" t="s">
         <v>96</v>
       </c>
@@ -2102,7 +2152,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A99" s="2" t="s">
         <v>97</v>
       </c>
@@ -2110,7 +2160,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A100" s="2" t="s">
         <v>98</v>
       </c>
@@ -2118,7 +2168,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A101" s="2" t="s">
         <v>99</v>
       </c>
@@ -2126,7 +2176,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A102" s="2" t="s">
         <v>100</v>
       </c>
@@ -2134,7 +2184,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A103" s="2" t="s">
         <v>101</v>
       </c>
@@ -2142,7 +2192,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A104" s="2" t="s">
         <v>102</v>
       </c>
@@ -2150,7 +2200,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A105" s="2" t="s">
         <v>103</v>
       </c>
@@ -2158,7 +2208,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A106" s="2" t="s">
         <v>104</v>
       </c>
@@ -2166,7 +2216,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A107" s="2" t="s">
         <v>105</v>
       </c>
@@ -2174,7 +2224,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A108" s="2" t="s">
         <v>106</v>
       </c>
@@ -2182,7 +2232,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A109" s="2" t="s">
         <v>107</v>
       </c>
@@ -2190,7 +2240,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A110" s="2" t="s">
         <v>108</v>
       </c>
@@ -2198,7 +2248,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A111" s="2" t="s">
         <v>109</v>
       </c>
@@ -2206,7 +2256,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A112" s="2" t="s">
         <v>110</v>
       </c>
@@ -2214,7 +2264,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A113" s="2" t="s">
         <v>111</v>
       </c>
@@ -2222,7 +2272,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A114" s="2" t="s">
         <v>112</v>
       </c>
@@ -2230,7 +2280,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A115" s="2" t="s">
         <v>113</v>
       </c>
@@ -2238,7 +2288,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A116" s="2" t="s">
         <v>114</v>
       </c>
@@ -2246,7 +2296,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A117" s="2" t="s">
         <v>115</v>
       </c>
@@ -2254,7 +2304,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A118" s="2" t="s">
         <v>116</v>
       </c>
@@ -2262,7 +2312,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A119" s="2" t="s">
         <v>117</v>
       </c>
@@ -2270,7 +2320,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A120" s="2" t="s">
         <v>118</v>
       </c>
@@ -2278,7 +2328,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A121" s="2" t="s">
         <v>119</v>
       </c>
@@ -2286,7 +2336,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A122" s="2" t="s">
         <v>120</v>
       </c>
@@ -2294,7 +2344,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A123" s="2" t="s">
         <v>121</v>
       </c>
@@ -2302,7 +2352,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A124" s="2" t="s">
         <v>122</v>
       </c>
@@ -2310,7 +2360,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A125" s="2" t="s">
         <v>123</v>
       </c>
@@ -2318,7 +2368,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A126" s="2" t="s">
         <v>124</v>
       </c>
@@ -2326,7 +2376,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A127" s="2" t="s">
         <v>125</v>
       </c>
@@ -2334,7 +2384,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A128" s="2" t="s">
         <v>126</v>
       </c>
@@ -2342,7 +2392,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A129" s="2" t="s">
         <v>127</v>
       </c>
@@ -2350,7 +2400,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A130" s="2" t="s">
         <v>128</v>
       </c>
@@ -2358,7 +2408,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A131" s="2" t="s">
         <v>129</v>
       </c>
@@ -2366,7 +2416,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A132" s="2" t="s">
         <v>130</v>
       </c>
@@ -2374,7 +2424,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A133" s="2" t="s">
         <v>131</v>
       </c>
@@ -2382,7 +2432,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A134" s="2" t="s">
         <v>132</v>
       </c>
@@ -2390,7 +2440,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A135" s="2" t="s">
         <v>133</v>
       </c>
@@ -2398,7 +2448,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A136" s="2" t="s">
         <v>134</v>
       </c>
@@ -2406,7 +2456,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A137" s="2" t="s">
         <v>135</v>
       </c>
@@ -2414,7 +2464,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A138" s="2" t="s">
         <v>136</v>
       </c>
@@ -2422,7 +2472,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A139" s="2" t="s">
         <v>137</v>
       </c>
@@ -2430,7 +2480,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A140" s="2" t="s">
         <v>138</v>
       </c>
@@ -2438,7 +2488,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A141" s="2" t="s">
         <v>139</v>
       </c>
@@ -2446,7 +2496,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A142" s="2" t="s">
         <v>140</v>
       </c>
@@ -2454,7 +2504,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A143" s="2" t="s">
         <v>141</v>
       </c>
@@ -2462,7 +2512,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A144" s="2" t="s">
         <v>142</v>
       </c>
@@ -2470,7 +2520,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A145" s="2" t="s">
         <v>143</v>
       </c>
@@ -2478,7 +2528,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A146" s="2" t="s">
         <v>144</v>
       </c>
@@ -2486,7 +2536,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A147" s="2" t="s">
         <v>145</v>
       </c>
@@ -2494,7 +2544,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A148" s="2" t="s">
         <v>146</v>
       </c>
@@ -2502,7 +2552,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A149" s="2" t="s">
         <v>147</v>
       </c>
@@ -2510,7 +2560,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A150" s="2" t="s">
         <v>148</v>
       </c>
@@ -2518,7 +2568,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A151" s="2" t="s">
         <v>149</v>
       </c>
@@ -2526,7 +2576,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A152" s="2" t="s">
         <v>150</v>
       </c>
@@ -2534,7 +2584,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A153" s="2" t="s">
         <v>151</v>
       </c>
@@ -2542,7 +2592,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A154" s="2" t="s">
         <v>152</v>
       </c>
@@ -2550,7 +2600,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A155" s="2" t="s">
         <v>153</v>
       </c>
@@ -2558,7 +2608,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A156" s="2" t="s">
         <v>154</v>
       </c>
@@ -2566,7 +2616,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A157" s="2" t="s">
         <v>155</v>
       </c>
@@ -2574,7 +2624,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A158" s="2" t="s">
         <v>156</v>
       </c>
@@ -2582,7 +2632,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A159" s="2" t="s">
         <v>157</v>
       </c>
@@ -2590,7 +2640,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A160" s="2" t="s">
         <v>158</v>
       </c>
@@ -2598,7 +2648,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="161" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A161" s="2" t="s">
         <v>159</v>
       </c>
@@ -2606,7 +2656,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="162" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A162" s="2" t="s">
         <v>160</v>
       </c>
@@ -2614,7 +2664,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A163" s="2" t="s">
         <v>161</v>
       </c>
@@ -2622,7 +2672,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A164" s="2" t="s">
         <v>162</v>
       </c>
@@ -2630,7 +2680,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A165" s="2" t="s">
         <v>163</v>
       </c>
@@ -2638,7 +2688,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A166" s="2" t="s">
         <v>164</v>
       </c>
@@ -2646,7 +2696,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="167" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A167" s="2" t="s">
         <v>165</v>
       </c>
@@ -2654,7 +2704,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="168" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A168" s="2" t="s">
         <v>166</v>
       </c>
@@ -2662,7 +2712,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="169" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A169" s="2" t="s">
         <v>167</v>
       </c>
@@ -2670,7 +2720,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="170" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A170" s="2" t="s">
         <v>168</v>
       </c>
@@ -2678,7 +2728,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="171" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A171" s="2" t="s">
         <v>169</v>
       </c>
@@ -2686,7 +2736,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="172" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A172" s="2" t="s">
         <v>170</v>
       </c>
@@ -2694,7 +2744,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="173" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A173" s="2" t="s">
         <v>171</v>
       </c>
@@ -2702,7 +2752,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="174" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A174" s="2" t="s">
         <v>172</v>
       </c>
@@ -2710,7 +2760,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="175" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A175" s="2" t="s">
         <v>173</v>
       </c>
@@ -2718,7 +2768,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="176" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A176" s="2" t="s">
         <v>174</v>
       </c>
@@ -2726,7 +2776,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="177" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A177" s="2" t="s">
         <v>175</v>
       </c>
@@ -2734,7 +2784,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="178" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A178" s="2" t="s">
         <v>176</v>
       </c>
@@ -2742,7 +2792,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="179" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A179" s="2" t="s">
         <v>177</v>
       </c>
@@ -2750,7 +2800,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="180" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A180" s="2" t="s">
         <v>178</v>
       </c>
@@ -2758,7 +2808,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="181" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A181" s="2" t="s">
         <v>179</v>
       </c>
@@ -2766,7 +2816,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="182" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A182" s="2" t="s">
         <v>180</v>
       </c>
@@ -2774,7 +2824,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="183" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A183" s="2" t="s">
         <v>181</v>
       </c>
@@ -2782,7 +2832,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="184" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A184" s="2" t="s">
         <v>182</v>
       </c>
@@ -2790,7 +2840,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="185" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A185" s="2" t="s">
         <v>183</v>
       </c>
@@ -2798,7 +2848,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="186" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A186" s="2" t="s">
         <v>184</v>
       </c>
@@ -2806,7 +2856,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="187" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A187" s="2" t="s">
         <v>185</v>
       </c>
@@ -2814,7 +2864,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="188" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A188" s="2" t="s">
         <v>186</v>
       </c>
@@ -2822,7 +2872,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="189" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A189" s="2" t="s">
         <v>187</v>
       </c>
@@ -2830,7 +2880,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="190" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A190" s="2" t="s">
         <v>188</v>
       </c>
@@ -2838,7 +2888,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="191" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A191" s="2" t="s">
         <v>189</v>
       </c>
@@ -2846,7 +2896,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="192" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A192" s="2" t="s">
         <v>190</v>
       </c>
@@ -2854,7 +2904,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="193" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A193" s="2" t="s">
         <v>191</v>
       </c>
@@ -2862,7 +2912,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="194" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A194" s="2" t="s">
         <v>192</v>
       </c>
@@ -2870,7 +2920,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="195" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A195" s="2" t="s">
         <v>193</v>
       </c>
@@ -2878,7 +2928,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="196" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A196" s="2" t="s">
         <v>194</v>
       </c>
@@ -2886,7 +2936,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="197" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A197" s="2" t="s">
         <v>195</v>
       </c>
@@ -2894,7 +2944,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="198" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A198" s="2" t="s">
         <v>196</v>
       </c>
@@ -2902,7 +2952,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="199" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A199" s="2" t="s">
         <v>197</v>
       </c>
@@ -2910,7 +2960,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="200" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A200" s="2" t="s">
         <v>198</v>
       </c>
@@ -2918,7 +2968,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="201" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A201" s="2" t="s">
         <v>199</v>
       </c>
@@ -2926,7 +2976,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="202" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A202" s="2" t="s">
         <v>200</v>
       </c>
@@ -2934,7 +2984,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="203" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A203" s="2" t="s">
         <v>201</v>
       </c>
@@ -2942,7 +2992,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="204" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A204" s="2" t="s">
         <v>202</v>
       </c>
@@ -2950,7 +3000,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="205" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A205" s="2" t="s">
         <v>203</v>
       </c>
@@ -2958,7 +3008,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="206" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A206" s="2" t="s">
         <v>204</v>
       </c>
@@ -2966,7 +3016,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="207" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A207" s="2" t="s">
         <v>205</v>
       </c>
@@ -2974,7 +3024,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="208" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A208" s="2" t="s">
         <v>206</v>
       </c>
@@ -2982,7 +3032,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="209" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A209" s="2" t="s">
         <v>207</v>
       </c>
@@ -2990,7 +3040,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="210" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A210" s="2" t="s">
         <v>208</v>
       </c>
@@ -2998,7 +3048,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="211" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A211" s="2" t="s">
         <v>209</v>
       </c>
@@ -3006,7 +3056,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="212" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A212" s="2" t="s">
         <v>210</v>
       </c>
@@ -3014,7 +3064,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="213" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A213" s="2" t="s">
         <v>211</v>
       </c>
@@ -3022,7 +3072,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="214" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A214" s="2" t="s">
         <v>212</v>
       </c>
@@ -3030,7 +3080,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="215" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A215" s="2" t="s">
         <v>213</v>
       </c>
@@ -3038,7 +3088,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="216" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A216" s="2" t="s">
         <v>214</v>
       </c>
@@ -3046,7 +3096,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="217" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A217" s="2" t="s">
         <v>215</v>
       </c>
@@ -3054,7 +3104,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="218" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A218" s="2" t="s">
         <v>216</v>
       </c>
@@ -3062,7 +3112,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="219" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A219" s="2" t="s">
         <v>217</v>
       </c>
@@ -3070,7 +3120,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="220" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A220" s="2" t="s">
         <v>218</v>
       </c>
@@ -3078,7 +3128,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="221" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A221" s="2" t="s">
         <v>219</v>
       </c>
@@ -3086,7 +3136,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="222" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A222" s="2" t="s">
         <v>220</v>
       </c>
@@ -3094,7 +3144,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="223" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A223" s="2" t="s">
         <v>221</v>
       </c>
@@ -3102,7 +3152,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="224" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A224" s="2" t="s">
         <v>222</v>
       </c>
@@ -3110,7 +3160,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="225" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A225" s="2" t="s">
         <v>223</v>
       </c>
@@ -3118,7 +3168,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="226" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A226" s="2" t="s">
         <v>224</v>
       </c>
@@ -3126,7 +3176,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="227" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A227" s="2" t="s">
         <v>225</v>
       </c>
@@ -3134,7 +3184,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="228" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A228" s="2" t="s">
         <v>226</v>
       </c>
@@ -3142,7 +3192,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="229" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A229" s="2" t="s">
         <v>227</v>
       </c>
@@ -3150,7 +3200,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="230" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A230" s="2" t="s">
         <v>228</v>
       </c>
@@ -3158,7 +3208,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="231" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A231" s="2" t="s">
         <v>229</v>
       </c>
@@ -3166,7 +3216,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="232" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A232" s="2" t="s">
         <v>230</v>
       </c>
@@ -3174,7 +3224,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="233" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A233" s="2" t="s">
         <v>231</v>
       </c>
@@ -3182,7 +3232,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="234" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A234" s="2" t="s">
         <v>232</v>
       </c>
@@ -3190,7 +3240,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="235" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A235" s="2" t="s">
         <v>233</v>
       </c>
@@ -3198,7 +3248,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="236" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A236" s="2" t="s">
         <v>234</v>
       </c>
@@ -3206,7 +3256,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="237" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A237" s="2" t="s">
         <v>235</v>
       </c>
@@ -3214,7 +3264,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="238" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A238" s="2" t="s">
         <v>236</v>
       </c>
@@ -3222,7 +3272,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="239" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A239" s="2" t="s">
         <v>237</v>
       </c>
@@ -3230,7 +3280,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="240" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A240" s="2" t="s">
         <v>238</v>
       </c>
@@ -3238,7 +3288,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="241" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A241" s="2" t="s">
         <v>239</v>
       </c>
@@ -3246,7 +3296,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="242" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A242" s="2" t="s">
         <v>240</v>
       </c>
@@ -3254,7 +3304,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="243" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A243" s="2" t="s">
         <v>241</v>
       </c>
@@ -3262,7 +3312,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="244" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A244" s="2" t="s">
         <v>242</v>
       </c>
@@ -3270,7 +3320,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="245" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A245" s="2" t="s">
         <v>243</v>
       </c>
@@ -3278,7 +3328,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="246" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A246" s="2" t="s">
         <v>244</v>
       </c>
@@ -3286,7 +3336,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="247" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A247" s="2" t="s">
         <v>245</v>
       </c>
@@ -3294,7 +3344,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="248" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A248" s="2" t="s">
         <v>246</v>
       </c>
@@ -3302,7 +3352,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="249" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A249" s="2" t="s">
         <v>247</v>
       </c>
@@ -3310,7 +3360,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="250" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A250" s="2" t="s">
         <v>248</v>
       </c>
@@ -3318,7 +3368,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="251" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A251" s="2" t="s">
         <v>249</v>
       </c>
@@ -3326,7 +3376,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="252" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A252" s="2" t="s">
         <v>250</v>
       </c>
@@ -3334,7 +3384,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="253" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A253" s="2" t="s">
         <v>251</v>
       </c>
@@ -3342,7 +3392,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="254" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A254" s="2" t="s">
         <v>252</v>
       </c>
@@ -3350,7 +3400,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="255" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A255" s="2" t="s">
         <v>253</v>
       </c>
@@ -3358,7 +3408,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="256" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A256" s="2" t="s">
         <v>254</v>
       </c>
@@ -3366,7 +3416,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="257" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A257" s="2" t="s">
         <v>255</v>
       </c>
@@ -3374,7 +3424,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="258" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A258" s="2" t="s">
         <v>256</v>
       </c>
@@ -3382,7 +3432,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="259" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A259" s="2" t="s">
         <v>257</v>
       </c>
@@ -3390,7 +3440,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="260" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A260" s="2" t="s">
         <v>258</v>
       </c>
@@ -3398,7 +3448,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="261" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A261" s="2" t="s">
         <v>259</v>
       </c>
@@ -3406,7 +3456,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="262" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A262" s="2" t="s">
         <v>260</v>
       </c>
@@ -3414,7 +3464,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="263" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A263" s="2" t="s">
         <v>261</v>
       </c>
@@ -3422,7 +3472,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="264" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A264" s="2" t="s">
         <v>262</v>
       </c>
@@ -3430,7 +3480,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="265" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A265" s="2" t="s">
         <v>263</v>
       </c>
@@ -3438,7 +3488,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="266" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A266" s="2" t="s">
         <v>264</v>
       </c>
@@ -3446,7 +3496,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="267" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A267" s="2" t="s">
         <v>265</v>
       </c>
@@ -3454,7 +3504,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="268" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A268" s="2" t="s">
         <v>266</v>
       </c>
@@ -3462,7 +3512,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="269" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A269" s="2" t="s">
         <v>267</v>
       </c>
@@ -3470,7 +3520,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="270" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A270" s="2" t="s">
         <v>268</v>
       </c>
@@ -3478,7 +3528,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="271" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A271" s="2" t="s">
         <v>269</v>
       </c>
@@ -3486,7 +3536,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="272" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A272" s="2" t="s">
         <v>270</v>
       </c>
@@ -3494,7 +3544,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="273" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A273" s="2" t="s">
         <v>271</v>
       </c>
@@ -3502,7 +3552,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="274" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A274" s="2" t="s">
         <v>272</v>
       </c>
@@ -3510,7 +3560,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="275" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A275" s="2" t="s">
         <v>273</v>
       </c>
@@ -3518,7 +3568,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="276" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A276" s="2" t="s">
         <v>274</v>
       </c>
@@ -3526,7 +3576,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="277" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A277" s="2" t="s">
         <v>275</v>
       </c>
@@ -3534,7 +3584,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="278" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A278" s="2" t="s">
         <v>276</v>
       </c>
@@ -3542,7 +3592,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="279" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A279" s="2" t="s">
         <v>277</v>
       </c>
@@ -3550,7 +3600,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="280" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A280" s="2" t="s">
         <v>278</v>
       </c>
@@ -3558,7 +3608,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="281" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A281" s="2" t="s">
         <v>279</v>
       </c>
@@ -3566,7 +3616,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="282" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A282" s="2" t="s">
         <v>280</v>
       </c>
@@ -3574,7 +3624,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="283" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A283" s="2" t="s">
         <v>281</v>
       </c>
@@ -3582,7 +3632,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="284" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A284" s="2" t="s">
         <v>282</v>
       </c>
@@ -3590,7 +3640,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="285" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A285" s="2" t="s">
         <v>283</v>
       </c>
@@ -3598,7 +3648,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="286" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A286" s="2" t="s">
         <v>284</v>
       </c>
@@ -3606,7 +3656,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="287" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A287" s="2" t="s">
         <v>285</v>
       </c>
@@ -3614,7 +3664,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="288" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A288" s="2" t="s">
         <v>286</v>
       </c>
@@ -3622,7 +3672,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="289" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A289" s="2" t="s">
         <v>287</v>
       </c>
@@ -3630,7 +3680,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="290" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A290" s="2" t="s">
         <v>288</v>
       </c>
@@ -3638,7 +3688,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="291" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A291" s="2" t="s">
         <v>289</v>
       </c>
@@ -3646,7 +3696,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="292" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A292" s="2" t="s">
         <v>290</v>
       </c>
@@ -3654,7 +3704,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="293" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A293" s="2" t="s">
         <v>291</v>
       </c>
@@ -3662,7 +3712,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="294" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A294" s="2" t="s">
         <v>292</v>
       </c>
@@ -3670,7 +3720,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="295" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A295" s="2" t="s">
         <v>293</v>
       </c>
@@ -3678,7 +3728,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="296" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A296" s="2" t="s">
         <v>294</v>
       </c>
@@ -3686,7 +3736,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="297" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A297" s="2" t="s">
         <v>295</v>
       </c>
@@ -3694,7 +3744,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="298" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A298" s="2" t="s">
         <v>296</v>
       </c>
@@ -3702,7 +3752,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="299" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A299" s="2" t="s">
         <v>297</v>
       </c>
@@ -3710,12 +3760,137 @@
         <v>301</v>
       </c>
     </row>
-    <row r="300" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A300" s="2" t="s">
         <v>298</v>
       </c>
       <c r="B300" s="3" t="s">
         <v>301</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{358332B7-B1BE-4E4E-BFC1-C30F55CDF54E}">
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="23.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>302</v>
+      </c>
+      <c r="B2" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>304</v>
+      </c>
+      <c r="B3" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>305</v>
+      </c>
+      <c r="B4" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>306</v>
+      </c>
+      <c r="B5" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>307</v>
+      </c>
+      <c r="B6" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>308</v>
+      </c>
+      <c r="B7" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>309</v>
+      </c>
+      <c r="B8" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="B9" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="B10" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="B11" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="B12" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>314</v>
+      </c>
+      <c r="B13" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="B14" t="s">
+        <v>303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>